<commit_message>
se actualiza archivos , desde assus 04_05-2026
</commit_message>
<xml_diff>
--- a/Estudiantes Pres vs Control acceso/Formato Objetos Transporte Control Acceso.xlsx
+++ b/Estudiantes Pres vs Control acceso/Formato Objetos Transporte Control Acceso.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\Estudiantes Pres vs Control acceso\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea\Documents\Backup_2026\Estudiantes Pres vs Control acceso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3505A0B7-9325-464E-9E60-DD49CBB7B622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="Objetos" sheetId="1" r:id="rId1"/>
@@ -172,8 +171,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,19 +610,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED66D76B-AB7C-48E0-8218-0FCDF9992D65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F95"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="37.5703125" customWidth="1"/>
-    <col min="2" max="2" width="47.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="37.625" customWidth="1"/>
+    <col min="2" max="2" width="47.375" customWidth="1"/>
+    <col min="3" max="3" width="19.125" customWidth="1"/>
+    <col min="4" max="4" width="16.375" style="4" customWidth="1"/>
     <col min="5" max="5" width="34" style="5" customWidth="1"/>
-    <col min="6" max="6" width="69.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="69.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -643,7 +642,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -665,7 +664,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -687,7 +686,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -709,7 +708,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -731,7 +730,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -753,7 +752,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -775,7 +774,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="D8" s="4" t="str">
         <f>IFERROR(VLOOKUP(C8,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -785,7 +784,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="D9" s="4" t="str">
         <f>IFERROR(VLOOKUP(C9,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -795,7 +794,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="D10" s="4" t="str">
         <f>IFERROR(VLOOKUP(C10,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -805,7 +804,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="B11" s="6"/>
       <c r="D11" s="4" t="str">
         <f>IFERROR(VLOOKUP(C11,listas!$A$2:$B$8,2,0),"")</f>
@@ -816,7 +815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="D12" s="4" t="str">
         <f>IFERROR(VLOOKUP(C12,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -826,7 +825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="D13" s="4" t="str">
         <f>IFERROR(VLOOKUP(C13,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -836,7 +835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="D14" s="4" t="str">
         <f>IFERROR(VLOOKUP(C14,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -846,7 +845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="D15" s="4" t="str">
         <f>IFERROR(VLOOKUP(C15,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -856,7 +855,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="D16" s="4" t="str">
         <f>IFERROR(VLOOKUP(C16,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -866,7 +865,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:5">
       <c r="D17" s="4" t="str">
         <f>IFERROR(VLOOKUP(C17,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -876,7 +875,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:5">
       <c r="D18" s="4" t="str">
         <f>IFERROR(VLOOKUP(C18,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -886,7 +885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:5">
       <c r="D19" s="4" t="str">
         <f>IFERROR(VLOOKUP(C19,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -896,7 +895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:5">
       <c r="D20" s="4" t="str">
         <f>IFERROR(VLOOKUP(C20,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -906,7 +905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:5">
       <c r="D21" s="4" t="str">
         <f>IFERROR(VLOOKUP(C21,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -916,7 +915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="22" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:5">
       <c r="D22" s="4" t="str">
         <f>IFERROR(VLOOKUP(C22,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -926,7 +925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:5">
       <c r="D23" s="4" t="str">
         <f>IFERROR(VLOOKUP(C23,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -936,7 +935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="24" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:5">
       <c r="D24" s="4" t="str">
         <f>IFERROR(VLOOKUP(C24,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -946,7 +945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="25" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:5">
       <c r="D25" s="4" t="str">
         <f>IFERROR(VLOOKUP(C25,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -956,7 +955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="26" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:5">
       <c r="D26" s="4" t="str">
         <f>IFERROR(VLOOKUP(C26,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -966,7 +965,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="27" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:5">
       <c r="D27" s="4" t="str">
         <f>IFERROR(VLOOKUP(C27,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -976,7 +975,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="28" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:5">
       <c r="D28" s="4" t="str">
         <f>IFERROR(VLOOKUP(C28,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -986,7 +985,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="29" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:5">
       <c r="D29" s="4" t="str">
         <f>IFERROR(VLOOKUP(C29,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -996,7 +995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="30" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:5">
       <c r="D30" s="4" t="str">
         <f>IFERROR(VLOOKUP(C30,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1006,7 +1005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="31" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:5">
       <c r="D31" s="4" t="str">
         <f>IFERROR(VLOOKUP(C31,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1016,7 +1015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="32" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:5">
       <c r="D32" s="4" t="str">
         <f>IFERROR(VLOOKUP(C32,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1026,7 +1025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="4:5">
       <c r="D33" s="4" t="str">
         <f>IFERROR(VLOOKUP(C33,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1036,7 +1035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="4:5">
       <c r="D34" s="4" t="str">
         <f>IFERROR(VLOOKUP(C34,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1046,7 +1045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="4:5">
       <c r="D35" s="4" t="str">
         <f>IFERROR(VLOOKUP(C35,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1056,7 +1055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:5">
       <c r="D36" s="4" t="str">
         <f>IFERROR(VLOOKUP(C36,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1066,7 +1065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="4:5">
       <c r="D37" s="4" t="str">
         <f>IFERROR(VLOOKUP(C37,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1076,7 +1075,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:5">
       <c r="D38" s="4" t="str">
         <f>IFERROR(VLOOKUP(C38,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1086,7 +1085,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="4:5">
       <c r="D39" s="4" t="str">
         <f>IFERROR(VLOOKUP(C39,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1096,7 +1095,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="40" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:5">
       <c r="D40" s="4" t="str">
         <f>IFERROR(VLOOKUP(C40,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1106,7 +1105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="4:5">
       <c r="D41" s="4" t="str">
         <f>IFERROR(VLOOKUP(C41,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1116,7 +1115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:5">
       <c r="D42" s="4" t="str">
         <f>IFERROR(VLOOKUP(C42,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1126,7 +1125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:5">
       <c r="D43" s="4" t="str">
         <f>IFERROR(VLOOKUP(C43,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1136,7 +1135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="4:5">
       <c r="D44" s="4" t="str">
         <f>IFERROR(VLOOKUP(C44,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1146,7 +1145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:5">
       <c r="D45" s="4" t="str">
         <f>IFERROR(VLOOKUP(C45,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1156,7 +1155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:5">
       <c r="D46" s="4" t="str">
         <f>IFERROR(VLOOKUP(C46,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1166,7 +1165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:5">
       <c r="D47" s="4" t="str">
         <f>IFERROR(VLOOKUP(C47,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1176,7 +1175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:5">
       <c r="D48" s="4" t="str">
         <f>IFERROR(VLOOKUP(C48,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1186,7 +1185,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="49" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:5">
       <c r="D49" s="4" t="str">
         <f>IFERROR(VLOOKUP(C49,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1196,7 +1195,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="50" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:5">
       <c r="D50" s="4" t="str">
         <f>IFERROR(VLOOKUP(C50,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1206,7 +1205,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="51" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:5">
       <c r="D51" s="4" t="str">
         <f>IFERROR(VLOOKUP(C51,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1216,7 +1215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="52" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:5">
       <c r="D52" s="4" t="str">
         <f>IFERROR(VLOOKUP(C52,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1226,7 +1225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="53" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:5">
       <c r="D53" s="4" t="str">
         <f>IFERROR(VLOOKUP(C53,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1236,7 +1235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="54" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:5">
       <c r="D54" s="4" t="str">
         <f>IFERROR(VLOOKUP(C54,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1246,7 +1245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="55" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:5">
       <c r="D55" s="4" t="str">
         <f>IFERROR(VLOOKUP(C55,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1256,7 +1255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="56" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="4:5">
       <c r="D56" s="4" t="str">
         <f>IFERROR(VLOOKUP(C56,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1266,7 +1265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="57" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="4:5">
       <c r="D57" s="4" t="str">
         <f>IFERROR(VLOOKUP(C57,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1276,7 +1275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="58" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="4:5">
       <c r="D58" s="4" t="str">
         <f>IFERROR(VLOOKUP(C58,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1286,7 +1285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="59" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="4:5">
       <c r="D59" s="4" t="str">
         <f>IFERROR(VLOOKUP(C59,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1296,7 +1295,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="4:5">
       <c r="D60" s="4" t="str">
         <f>IFERROR(VLOOKUP(C60,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1306,7 +1305,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="4:5">
       <c r="D61" s="4" t="str">
         <f>IFERROR(VLOOKUP(C61,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1316,7 +1315,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="4:5">
       <c r="D62" s="4" t="str">
         <f>IFERROR(VLOOKUP(C62,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1326,7 +1325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="4:5">
       <c r="D63" s="4" t="str">
         <f>IFERROR(VLOOKUP(C63,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1336,7 +1335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="4:5">
       <c r="D64" s="4" t="str">
         <f>IFERROR(VLOOKUP(C64,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1346,7 +1345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:5">
       <c r="D65" s="4" t="str">
         <f>IFERROR(VLOOKUP(C65,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1356,7 +1355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:5">
       <c r="D66" s="4" t="str">
         <f>IFERROR(VLOOKUP(C66,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1366,7 +1365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:5">
       <c r="D67" s="4" t="str">
         <f>IFERROR(VLOOKUP(C67,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1376,7 +1375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="4:5">
       <c r="D68" s="4" t="str">
         <f>IFERROR(VLOOKUP(C68,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1386,7 +1385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="4:5">
       <c r="D69" s="4" t="str">
         <f>IFERROR(VLOOKUP(C69,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1396,7 +1395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="4:5">
       <c r="D70" s="4" t="str">
         <f>IFERROR(VLOOKUP(C70,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1406,7 +1405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="4:5">
       <c r="D71" s="4" t="str">
         <f>IFERROR(VLOOKUP(C71,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1416,7 +1415,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="4:5">
       <c r="D72" s="4" t="str">
         <f>IFERROR(VLOOKUP(C72,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1426,7 +1425,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="4:5">
       <c r="D73" s="4" t="str">
         <f>IFERROR(VLOOKUP(C73,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1436,7 +1435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="4:5">
       <c r="D74" s="4" t="str">
         <f>IFERROR(VLOOKUP(C74,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1446,7 +1445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="4:5">
       <c r="D75" s="4" t="str">
         <f>IFERROR(VLOOKUP(C75,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1456,7 +1455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="4:5">
       <c r="D76" s="4" t="str">
         <f>IFERROR(VLOOKUP(C76,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1466,7 +1465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="4:5">
       <c r="D77" s="4" t="str">
         <f>IFERROR(VLOOKUP(C77,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1476,7 +1475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="4:5">
       <c r="D78" s="4" t="str">
         <f>IFERROR(VLOOKUP(C78,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1486,7 +1485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="4:5">
       <c r="D79" s="4" t="str">
         <f>IFERROR(VLOOKUP(C79,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1496,7 +1495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="4:5">
       <c r="D80" s="4" t="str">
         <f>IFERROR(VLOOKUP(C80,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1506,7 +1505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="4:5">
       <c r="D81" s="4" t="str">
         <f>IFERROR(VLOOKUP(C81,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1516,7 +1515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="4:5">
       <c r="D82" s="4" t="str">
         <f>IFERROR(VLOOKUP(C82,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1526,7 +1525,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="4:5">
       <c r="D83" s="4" t="str">
         <f>IFERROR(VLOOKUP(C83,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1536,7 +1535,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="4:5">
       <c r="D84" s="4" t="str">
         <f>IFERROR(VLOOKUP(C84,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1546,7 +1545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="4:5">
       <c r="D85" s="4" t="str">
         <f>IFERROR(VLOOKUP(C85,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1556,7 +1555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="4:5">
       <c r="D86" s="4" t="str">
         <f>IFERROR(VLOOKUP(C86,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1566,7 +1565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="4:5">
       <c r="D87" s="4" t="str">
         <f>IFERROR(VLOOKUP(C87,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1576,7 +1575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="4:5">
       <c r="D88" s="4" t="str">
         <f>IFERROR(VLOOKUP(C88,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1586,7 +1585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="4:5">
       <c r="D89" s="4" t="str">
         <f>IFERROR(VLOOKUP(C89,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1596,7 +1595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="4:5">
       <c r="D90" s="4" t="str">
         <f>IFERROR(VLOOKUP(C90,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1606,31 +1605,31 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="4:5">
       <c r="D91" s="4" t="str">
         <f>IFERROR(VLOOKUP(C91,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="92" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="4:5">
       <c r="D92" s="4" t="str">
         <f>IFERROR(VLOOKUP(C92,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="93" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="4:5">
       <c r="D93" s="4" t="str">
         <f>IFERROR(VLOOKUP(C93,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="94" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="4:5">
       <c r="D94" s="4" t="str">
         <f>IFERROR(VLOOKUP(C94,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="95" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="4:5">
       <c r="D95" s="4" t="str">
         <f>IFERROR(VLOOKUP(C95,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1638,7 +1637,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C15" xr:uid="{4E78058F-6DE9-4785-B4B6-576D9F0A6DEF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C15">
       <formula1>TIPO_OBJETO</formula1>
     </dataValidation>
   </dataValidations>
@@ -1647,19 +1646,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75E2AA2-5432-4E9C-93A9-C36766097F89}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="41.42578125" customWidth="1"/>
+    <col min="2" max="2" width="41.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="B1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1670,7 +1669,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1681,7 +1680,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1692,7 +1691,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1703,7 +1702,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1720,15 +1719,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6E318EA-3F07-4D83-8AAC-62F6B6937B60}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="36.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="36.125" customWidth="1"/>
+    <col min="2" max="2" width="23.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1736,7 +1735,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1744,7 +1743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1760,7 +1759,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1768,7 +1767,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1776,7 +1775,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1784,7 +1783,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>30</v>
       </c>

</xml_diff>